<commit_message>
Prioritize pip validator setup and update artifacts
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/text_comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/text_comparison.xlsx
@@ -842,15 +842,111 @@
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
+          <t>Le 3 février 2025, lors de la clôture de l'acquisition de CWB, la Banque a émis un total de 50 272 878 actions ordinaires, pour un produit brut de 6,3 G$.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>OUI — Nouvel élément à surveiller : Oui.
+Sujet détecté : Information ajoutée, capital réglementaire.
+Ce qui change : Le T2 ajoute des informations sur l'émission de 50 272 878 actions ordinaires pour un produit brut de 6,3 G$ lors de l'acquisition de CWB.
+Pertinence métier : Ce changement met l'accent sur l'évolution de la structure de capital de la banque suite à une acquisition majeure. L'émission d'actions ordinaires modifie la composition du capital réglementaire et peut influencer la perception de la solidité financière de la banque par les régulateurs et les investisseurs.
+Point de surveillance : Capital réglementaire — Le changement indique une augmentation du capital par émission d'actions, ce qui peut affecter les ratios de capital et la comparabilité avec les pairs.</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>c'et pas un vrai changement pas important vraiment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Activités de gestion</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Le 3 février 2025, dans le cadre de l'acquisition de CWB, la Banque a acquis les obligations liées aux dettes subordonnées de CWB pour un montant total de 525 M$, qui incluait une débenture de 125 M$ portant intérêt à 4,840 % et échéant le 29 juin 2030 (le 2 mai 2025, la Banque a informé les détenteurs de son intention de racheter les débentures le 29 juin 2025, à un prix de rachat égal au capital impayé plus l'intérêt couru et impayé), une débenture de 150 M$ portant intérêt à 5,937 % et échéant le 22 décembre 2032 et une débenture de 250 M$ portant intérêt à 5,949 % et échéant le 29 janvier 2034. Comme les débentures respectent les exigences relatives aux FPUNV, elles sont admissibles aux fins du calcul des fonds propres réglementaires selon les règles de Bâle III.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>OUI — Nouvel élément à surveiller : Oui.
+Sujet détecté : Information ajoutée, fonds propres réglementaires.
+Ce qui change : Le T2 ajoute des informations sur l'acquisition de 525 M$ d'obligations liées aux dettes subordonnées de CWB, incluant des débentures portant intérêt à des taux spécifiques.
+Pertinence métier : Ce changement met l'accent sur l'intégration de nouveaux instruments de fonds propres dans le calcul des fonds propres réglementaires. L'acquisition de ces obligations peut influencer la structure de capital de la banque et sa capacité à répondre aux exigences réglementaires.
+Point de surveillance : Fonds propres réglementaires — Le changement indique une modification de la composition des fonds propres, ce qui peut affecter les ratios de capital et la comparabilité avec les pairs.</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>oui une nouvelle idee mais vraiment pas pertinant quand meme pour nous</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Activités de gestion</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Ajout</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
           <t>Le 20 février 2025, il y a eu un échange de la totalité des actions privilégiées de premier rang, série 5 et série 9, émises et en circulation de CWB, contre des actions privilégiées de premier rang essentiellement équivalentes de la Banque Nationale, série 47 et série 49, donnant droit à un dividende non cumulatif à taux rajusté tous les cinq ans, portant intérêt à 6,371 % et 7,651 %. La Banque a échangé 10 000 000 actions privilégiées pour un montant total de 264 M$. Comme les actions privilégiées, série 47 et série 49, respectent les exigences relatives aux FPUNV, elles sont admissibles aux fins du calcul des fonds propres réglementaires selon les règles de Bâle III.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>OUI — Nouvel élément à surveiller : Oui.
 Sujet détecté : Information ajoutée, fonds propres réglementaires.
@@ -859,50 +955,258 @@
 Point de surveillance : Fonds propres réglementaires — Le changement indique une modification de la composition des fonds propres, ce qui peut affecter les ratios de capital et la comparabilité avec les pairs.</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Actions, autres instruments de capitaux propres et options d'achat d'actions</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Si un événement déclencheur faisant intervenir les clauses FPUNV devait se produire, toutes les actions privilégiées et les BCRL de la Banque ainsi que les billets à moyen terme échéant le 16 août 2032, le 15 février 2034 et le 15 février 2035, qui sont des instruments de fonds propres assortis d'une clause FPUNV, seraient convertis en actions ordinaires de la Banque selon une formule de conversion automatique, à un prix de conversion correspondant au plus élevé des montants suivants : i) un prix plancher contractuel de 5,00 $; ii) le cours du marché des actions ordinaires de la Banque à la date de l'événement déclencheur (cours moyen pondéré sur 10 jours).</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Si un événement déclencheur faisant intervenir les clauses FPUNV devait se produire, toutes les actions privilégiées et les BCRL de la Banque ainsi que les billets à moyen terme et les débentures subordonnées, qui sont des instruments de fonds propres assortis d'une clause FPUNV, seraient convertis en actions ordinaires de la Banque selon une formule de conversion automatique, à un prix de conversion correspondant au plus élevé des montants suivants : i) un prix plancher contractuel de 5,00 $; ii) le cours du marché des actions ordinaires de la Banque à la date de l'événement déclencheur (cours moyen pondéré sur 10 jours).</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>OUI — Nouvel élément à surveiller : Oui.
+Sujet détecté : Information ajoutée, fonds propres réglementaires.
+Ce qui change : Le T2 ajoute les débentures subordonnées à la liste des instruments convertibles en actions ordinaires en cas de déclenchement des clauses FPUNV.
+Pertinence métier : Ce changement met l'accent sur la transparence de la divulgation concernant les fonds propres réglementaires. L'ajout de ces débentures modifie la perception de la solidité financière de la banque et sa capacité à absorber les pertes en cas de crise.
+Point de surveillance : Fonds propres réglementaires — Le changement indique une modification de la composition des instruments convertibles, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Actif pondéré en fonction des risques selon les principaux facteurs de risque</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>L'actif pondéré en fonction des risques a augmenté de 7,5 G$ pour s'établir à 148,5 G$ au 31 janvier 2025, comparativement à 141,0 G$ au 31 octobre 2024. Cette augmentation découle principalement de la croissance organique de l'actif pondéré en fonction des risques, de la variation du taux de change et de la détérioration de la qualité de crédit du portefeuille de prêts. La variation de l'actif pondéré en fonction des risques de la Banque par type de risque est présentée dans le tableau suivant.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>L'actif pondéré en fonction des risques a augmenté de 41,8 G$ pour s'établir à 182,8 G$ au 30 avril 2025, comparativement à 141,0 G$ au 31 octobre 2024. Cette augmentation découle principalement de l'inclusion de CWB, ainsi que de la croissance organique de l'actif pondéré en fonction des risques et de la détérioration de la qualité de crédit du portefeuille de prêts. La variation de l'actif pondéré en fonction des risques de la Banque par type de risque est présentée dans le tableau suivant.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>OUI — Nouvel élément à surveiller : Oui.
+Sujet détecté : Texte de risque modifié, fonds propres réglementaires.
+Ce qui change : Le T2 ajoute l'inclusion de CWB comme facteur d'augmentation de l'actif pondéré en fonction des risques, absent au T1.
+Pertinence métier : Ce changement met l'accent sur l'évolution des facteurs influençant les ratios de capital de la banque. L'ajout de CWB modifie la perception de la solidité financière de la banque et sa capacité à répondre aux exigences réglementaires.
+Point de surveillance : Fonds propres réglementaires — Le changement indique une modification des facteurs influençant les ratios de capital, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Ratios des fonds propres réglementaires, de levier et TLAC</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Le ratio de levier en date du 31 janvier 2025 s'établit à 4,3 %, comparativement à 4,4 % au 31 octobre 2024. La baisse du ratio de levier s'explique essentiellement par l'augmentation de l'exposition totale, en partie contrebalancée par la croissance des fonds propres de catégorie 1.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Le ratio de levier en date du 30 avril 2025 s'établit à 4,7 %, comparativement à 4,4 % au 31 octobre 2024. L'augmentation du ratio de levier s'explique essentiellement par la croissance des fonds propres de catégorie 1 en lien avec les actions ordinaires émises dans le cadre de l'acquisition de CWB, en partie contrebalancée par l'augmentation de l'exposition totale.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>OUI — Nouvel élément à surveiller : Oui.
+Sujet détecté : Texte de risque modifié, ratio ou seuil prudentiel.
+Ce qui change : Le T2 ajoute l'acquisition de CWB comme facteur influençant le ratio de levier, absent au T1.
+Pertinence métier : Ce changement met l'accent sur l'évolution des facteurs influençant les ratios de capital de la banque. L'ajout de CWB modifie la perception de la solidité financière de la banque et sa capacité à répondre aux exigences réglementaires.
+Point de surveillance : Ratios réglementaires — Le changement indique une modification des facteurs influençant les ratios de capital, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Ratios des fonds propres réglementaires, de levier et TLAC</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Au 31 janvier 2025, le ratio TLAC et le ratio de levier TLAC s'établissent à 31,2 % et à 8,7 %, comparativement à 31,2 % et à 8,6 %, respectivement, au 31 octobre 2024. Le ratio TLAC est demeuré stable et l'augmentation du ratio de levier TLAC s'explique principalement par les émissions nettes d'instruments qui satisfont tous les critères d'admissibilité TLAC au cours du premier trimestre de 2025.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Au 30 avril 2025, le ratio TLAC et le ratio de levier TLAC s'établissent à 28,2 % et à 8,8 %, comparativement à 31,2 % et à 8,6 %, respectivement, au 31 octobre 2024. L'augmentation du ratio de levier TLAC s'explique principalement par les émissions nettes d'instruments qui satisfont tous les critères d'admissibilité TLAC au cours de la période. Cependant, la croissance de l'actif pondéré en fonction des risques, principalement attribuable à l'inclusion de CWB, a largement compensé ces émissions, ce qui a entraîné une diminution du ratio TLAC.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>OUI — Nouvel élément à surveiller : Oui.
+Sujet détecté : Texte de risque modifié, ratio ou seuil prudentiel.
+Ce qui change : Le T2 ajoute l'inclusion de CWB comme facteur influençant le ratio TLAC, absent au T1.
+Pertinence métier : Ce changement met l'accent sur l'évolution des facteurs influençant les ratios de capital de la banque. L'ajout de CWB modifie la perception de la solidité financière de la banque et sa capacité à répondre aux exigences réglementaires.
+Point de surveillance : Ratios réglementaires — Le changement indique une modification des facteurs influençant les ratios de capital, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Activités de gestion</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Le 17 février 2025, soit le premier jour ouvrable suivant la date de rachat du 15 février 2025, la Banque a terminé le rachat de la totalité des actions privilégiées de premier rang à dividende non cumulatif à taux rajusté tous les cinq ans, série 32, émises et en circulation. Tel que prévu dans les conditions relatives aux actions, le prix de rachat était de 25,00 $ l'action, plus les dividendes périodiques déclarés et impayés. La Banque a racheté 12 000 000 actions privilégiées série 32 pour un prix total de 300 M$. Ces instruments ont été exclus du calcul des ratios de fonds propres au 31 janvier 2025.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Le 17 février 2025, soit le premier jour ouvrable suivant la date de rachat du 15 février 2025, la Banque a terminé le rachat de la totalité des actions privilégiées de premier rang à dividende non cumulatif à taux rajusté tous les cinq ans, série 32, émises et en circulation. Tel que prévu dans les conditions relatives aux actions, le prix de rachat était de 25,00 $ l'action, plus les dividendes périodiques déclarés et impayés. La Banque a racheté 12 000 000 actions privilégiées série 32 pour un prix total de 300 M$.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>OUI — Nouvel élément à surveiller : Oui.
 Sujet détecté : Information retirée, fonds propres réglementaires.
@@ -911,313 +1215,9 @@
 Point de surveillance : Fonds propres réglementaires — Le changement indique une modification de la divulgation sur la composition des fonds propres, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>Non pas un vrai changement</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Actions, autres instruments de capitaux propres et options d'achat d'actions</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Si un événement déclencheur faisant intervenir les clauses FPUNV devait se produire, toutes les actions privilégiées et les BCRL de la Banque ainsi que les billets à moyen terme échéant le 16 août 2032, le 15 février 2034 et le 15 février 2035, qui sont des instruments de fonds propres assortis d'une clause FPUNV, seraient convertis en actions ordinaires de la Banque selon une formule de conversion automatique, à un prix de conversion correspondant au plus élevé des montants suivants : i) un prix plancher contractuel de 5,00 $; ii) le cours du marché des actions ordinaires de la Banque à la date de l'événement déclencheur (cours moyen pondéré sur 10 jours).</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Si un événement déclencheur faisant intervenir les clauses FPUNV devait se produire, toutes les actions privilégiées et les BCRL de la Banque ainsi que les billets à moyen terme et les débentures subordonnées, qui sont des instruments de fonds propres assortis d'une clause FPUNV, seraient convertis en actions ordinaires de la Banque selon une formule de conversion automatique, à un prix de conversion correspondant au plus élevé des montants suivants : i) un prix plancher contractuel de 5,00 $; ii) le cours du marché des actions ordinaires de la Banque à la date de l'événement déclencheur (cours moyen pondéré sur 10 jours).</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>OUI — Nouvel élément à surveiller : Oui.
-Sujet détecté : Information ajoutée, fonds propres réglementaires.
-Ce qui change : Le T2 ajoute les débentures subordonnées à la liste des instruments convertibles en actions ordinaires en cas de déclenchement des clauses FPUNV.
-Pertinence métier : Ce changement met l'accent sur la transparence de la divulgation concernant les fonds propres réglementaires. L'ajout de ces débentures modifie la perception de la solidité financière de la banque et sa capacité à absorber les pertes en cas de crise.
-Point de surveillance : Fonds propres réglementaires — Le changement indique une modification de la composition des instruments convertibles, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Actif pondéré en fonction des risques selon les principaux facteurs de risque</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>L'actif pondéré en fonction des risques a augmenté de 7,5 G$ pour s'établir à 148,5 G$ au 31 janvier 2025, comparativement à 141,0 G$ au 31 octobre 2024. Cette augmentation découle principalement de la croissance organique de l'actif pondéré en fonction des risques, de la variation du taux de change et de la détérioration de la qualité de crédit du portefeuille de prêts. La variation de l'actif pondéré en fonction des risques de la Banque par type de risque est présentée dans le tableau suivant.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>L'actif pondéré en fonction des risques a augmenté de 41,8 G$ pour s'établir à 182,8 G$ au 30 avril 2025, comparativement à 141,0 G$ au 31 octobre 2024. Cette augmentation découle principalement de l'inclusion de CWB, ainsi que de la croissance organique de l'actif pondéré en fonction des risques et de la détérioration de la qualité de crédit du portefeuille de prêts. La variation de l'actif pondéré en fonction des risques de la Banque par type de risque est présentée dans le tableau suivant.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>OUI — Nouvel élément à surveiller : Oui.
-Sujet détecté : Texte de risque modifié, fonds propres réglementaires.
-Ce qui change : Le T2 ajoute l'inclusion de CWB comme facteur d'augmentation de l'actif pondéré en fonction des risques, absent au T1.
-Pertinence métier : Ce changement met l'accent sur l'évolution des facteurs influençant les ratios de capital de la banque. L'ajout de CWB modifie la perception de la solidité financière de la banque et sa capacité à répondre aux exigences réglementaires.
-Point de surveillance : Fonds propres réglementaires — Le changement indique une modification des facteurs influençant les ratios de capital, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Ratios des fonds propres réglementaires, de levier et TLAC</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Le ratio de levier en date du 31 janvier 2025 s'établit à 4,3 %, comparativement à 4,4 % au 31 octobre 2024. La baisse du ratio de levier s'explique essentiellement par l'augmentation de l'exposition totale, en partie contrebalancée par la croissance des fonds propres de catégorie 1.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Le ratio de levier en date du 30 avril 2025 s'établit à 4,7 %, comparativement à 4,4 % au 31 octobre 2024. L'augmentation du ratio de levier s'explique essentiellement par la croissance des fonds propres de catégorie 1 en lien avec les actions ordinaires émises dans le cadre de l'acquisition de CWB, en partie contrebalancée par l'augmentation de l'exposition totale.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>OUI — Nouvel élément à surveiller : Oui.
-Sujet détecté : Texte de risque modifié, ratio ou seuil prudentiel.
-Ce qui change : Le T2 ajoute l'acquisition de CWB comme facteur influençant le ratio de levier, absent au T1.
-Pertinence métier : Ce changement met l'accent sur l'évolution des facteurs influençant les ratios de capital de la banque. L'ajout de CWB modifie la perception de la solidité financière de la banque et sa capacité à répondre aux exigences réglementaires.
-Point de surveillance : Ratios réglementaires — Le changement indique une modification des facteurs influençant les ratios de capital, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Ratios des fonds propres réglementaires, de levier et TLAC</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Au 31 janvier 2025, le ratio TLAC et le ratio de levier TLAC s'établissent à 31,2 % et à 8,7 %, comparativement à 31,2 % et à 8,6 %, respectivement, au 31 octobre 2024. Le ratio TLAC est demeuré stable et l'augmentation du ratio de levier TLAC s'explique principalement par les émissions nettes d'instruments qui satisfont tous les critères d'admissibilité TLAC au cours du premier trimestre de 2025.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Au 30 avril 2025, le ratio TLAC et le ratio de levier TLAC s'établissent à 28,2 % et à 8,8 %, comparativement à 31,2 % et à 8,6 %, respectivement, au 31 octobre 2024. L'augmentation du ratio de levier TLAC s'explique principalement par les émissions nettes d'instruments qui satisfont tous les critères d'admissibilité TLAC au cours de la période. Cependant, la croissance de l'actif pondéré en fonction des risques, principalement attribuable à l'inclusion de CWB, a largement compensé ces émissions, ce qui a entraîné une diminution du ratio TLAC.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>OUI — Nouvel élément à surveiller : Oui.
-Sujet détecté : Texte de risque modifié, ratio ou seuil prudentiel.
-Ce qui change : Le T2 ajoute l'inclusion de CWB comme facteur influençant le ratio TLAC, absent au T1.
-Pertinence métier : Ce changement met l'accent sur l'évolution des facteurs influençant les ratios de capital de la banque. L'ajout de CWB modifie la perception de la solidité financière de la banque et sa capacité à répondre aux exigences réglementaires.
-Point de surveillance : Ratios réglementaires — Le changement indique une modification des facteurs influençant les ratios de capital, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Activités de gestion</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Le 3 février 2025, lors de la clôture de l'acquisition de CWB, la Banque a émis un total de 50 272 878 actions ordinaires, pour un produit brut de 6,3 G$.</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>OUI — Nouvel élément à surveiller : Oui.
-Sujet détecté : Information ajoutée, capital réglementaire.
-Ce qui change : Le T2 ajoute des informations sur l'émission de 50 272 878 actions ordinaires pour un produit brut de 6,3 G$ lors de l'acquisition de CWB.
-Pertinence métier : Ce changement met l'accent sur l'évolution de la structure de capital de la banque suite à une acquisition majeure. L'émission d'actions ordinaires modifie la composition du capital réglementaire et peut influencer la perception de la solidité financière de la banque par les régulateurs et les investisseurs.
-Point de surveillance : Capital réglementaire — Le changement indique une augmentation du capital par émission d'actions, ce qui peut affecter les ratios de capital et la comparabilité avec les pairs.</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>c'et pas un vrai changement pas important vraiment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Gestion du capital</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Activités de gestion</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Ajout</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>Le 3 février 2025, dans le cadre de l'acquisition de CWB, la Banque a acquis les obligations liées aux dettes subordonnées de CWB pour un montant total de 525 M$, qui incluait une débenture de 125 M$ portant intérêt à 4,840 % et échéant le 29 juin 2030 (le 2 mai 2025, la Banque a informé les détenteurs de son intention de racheter les débentures le 29 juin 2025, à un prix de rachat égal au capital impayé plus l'intérêt couru et impayé), une débenture de 150 M$ portant intérêt à 5,937 % et échéant le 22 décembre 2032 et une débenture de 250 M$ portant intérêt à 5,949 % et échéant le 29 janvier 2034. Comme les débentures respectent les exigences relatives aux FPUNV, elles sont admissibles aux fins du calcul des fonds propres réglementaires selon les règles de Bâle III.</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>OUI — Nouvel élément à surveiller : Oui.
-Sujet détecté : Information ajoutée, fonds propres réglementaires.
-Ce qui change : Le T2 ajoute des informations sur l'acquisition de 525 M$ d'obligations liées aux dettes subordonnées de CWB, incluant des débentures portant intérêt à des taux spécifiques.
-Pertinence métier : Ce changement met l'accent sur l'intégration de nouveaux instruments de fonds propres dans le calcul des fonds propres réglementaires. L'acquisition de ces obligations peut influencer la structure de capital de la banque et sa capacité à répondre aux exigences réglementaires.
-Point de surveillance : Fonds propres réglementaires — Le changement indique une modification de la composition des fonds propres, ce qui peut affecter les ratios de capital et la comparabilité avec les pairs.</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>oui une nouvelle idee mais vraiment pas pertinant quand meme pour nous</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: extend risk triage for data cloud and third parties
</commit_message>
<xml_diff>
--- a/outputs/resultats/bnc/2025_t2_vs_2025_t1/text_comparison.xlsx
+++ b/outputs/resultats/bnc/2025_t2_vs_2025_t1/text_comparison.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyse complète" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analyse complète'!$A$1:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analyse complète'!$A$1:$J$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,7 +34,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +51,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00D6E4F0"/>
         <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADADD"/>
+        <bgColor rgb="00FADADD"/>
       </patternFill>
     </fill>
     <fill>
@@ -78,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -87,6 +93,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -457,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J28"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -623,38 +632,90 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Risque de marché</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Le risque de marché est le risque de pertes financières liées à la variation des prix de marché. La Banque est exposée au risque de marché en raison de sa participation à des activités de négociation, d'investissement et de gestion de l'appariement du bilan. Depuis quelques années, la Banque fait face à un contexte volatil. Le contexte géopolitique, notamment les mesures affectant les relations commerciales entre le Canada et ses partenaires, incluant l'imposition de tarifs et toute mesure de riposte, la guerre russo-ukrainienne ainsi que les affrontements entre Israël et le Hamas, l'inflation, les changements climatiques et les taux d'intérêt élevés continuent à créer des incertitudes.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Le risque de marché est le risque de pertes financières liées à la variation des prix de marché. La Banque est exposée au risque de marché en raison de sa participation à des activités de négociation, d'investissement et de gestion de l'appariement du bilan.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>OUI — Nouvel élément à surveiller : Oui.
+Sujet détecté : Texte de risque modifié, information retirée.
+Ce qui change : Le T2 retire la description du contexte géopolitique et économique volatile, incluant les mesures commerciales, la guerre russo-ukrainienne, et les affrontements entre Israël et le Hamas, qui étaient mentionnés au T1.
+Pertinence métier : Ce changement met l'accent sur l'évolution du cadre réglementaire applicable aux divulgations climatiques des institutions financières. La mise à jour de la ligne directrice B-15 par le BSIF, notamment le report des exigences liées aux émissions de GES de portée 3, peut influencer la manière dont les banques planifient leur conformité, structurent leurs contrôles ESG et communiquent leurs risques climatiques. Ce point est important à suivre, car il permet d'évaluer l'évolution des attentes prudentielles, la comparabilité des pratiques de divulgation entre pairs et le niveau de préparation des banques face aux exigences climatiques.
+Point de surveillance : Risque climatique / ESG — Le changement indique que la banque tient compte de la mise à jour de la ligne directrice B-15 du BSIF et du report des exigences liées aux émissions de GES de portée 3. Ce point permet de suivre l'adaptation des banques aux attentes prudentielles climatiques, leur niveau de préparation ESG et la comparabilité de leurs pratiques de divulgation entre pairs.</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Exigences de communication publique pour les banques d'importance systémique mondiale</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Suppression</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Le CBCB a développé une méthodologie d'évaluation et d'exigence de capacité additionnelle d'absorption des pertes ainsi que des indicateurs utilisés par le CBCB et le Conseil de stabilité financière pour évaluer les banques d'importance systémique mondiale (BISM). Des exigences de communication publique annuelles s'appliquent aux grandes banques actives à l'échelle mondiale.
 La dernière version du préavis du BSIF intitulé Banques d'importance systémique mondiale - Obligations redditionnelles à l'égard de la mise en œuvre des exigences de communication publique pour les BISM au Canada est entrée en vigueur en 2022. Les banques canadiennes, y compris la Banque, qui n'ont pas été désignées BISM et qui ont une exposition totale (telle que calculée par le ratio de levier selon Bâle III) supérieure à l'équivalent de 200 milliards d'euros à la fin de l'exercice sont tenues de publier annuellement les indicateurs. Les indicateurs sont calculés et présentés selon des lignes directrices précises publiées par le CBCB, qui sont mises à jour chaque année. Ainsi, les valeurs obtenues ne sont peut-être pas comparables aux autres mesures présentées dans ce rapport. Le tableau suivant présente les indicateurs utilisés dans la méthode d'évaluation du CBCB permettant d'évaluer les BISM.</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>OUI — Nouvel élément à surveiller : Oui.
 Sujet détecté : Information retirée, exigences réglementaires ou conformité.
@@ -663,63 +724,11 @@
 Point de surveillance : Exigences réglementaires — Le changement indique une modification de la divulgation sur les obligations de communication, ce qui peut affecter la comparabilité avec les pairs et la lecture des pratiques de conformité.</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Oui c'est un vrai changment</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Gestion des risques</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Risque de marché</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>33</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Le risque de marché est le risque de pertes financières liées à la variation des prix de marché. La Banque est exposée au risque de marché en raison de sa participation à des activités de négociation, d'investissement et de gestion de l'appariement du bilan. Depuis quelques années, la Banque fait face à un contexte volatil. Le contexte géopolitique, notamment les mesures affectant les relations commerciales entre le Canada et ses partenaires, incluant l'imposition de tarifs et toute mesure de riposte, la guerre russo-ukrainienne ainsi que les affrontements entre Israël et le Hamas, l'inflation, les changements climatiques et les taux d'intérêt élevés continuent à créer des incertitudes.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Le risque de marché est le risque de pertes financières liées à la variation des prix de marché. La Banque est exposée au risque de marché en raison de sa participation à des activités de négociation, d'investissement et de gestion de l'appariement du bilan.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>OUI — Nouvel élément à surveiller : Oui.
-Sujet détecté : Texte de risque modifié, information retirée.
-Ce qui change : Le T2 retire la description du contexte géopolitique et économique volatile, incluant les mesures commerciales, la guerre russo-ukrainienne, et les affrontements entre Israël et le Hamas, qui étaient mentionnés au T1.
-Pertinence métier : Ce changement met l'accent sur l'évolution du cadre réglementaire applicable aux divulgations climatiques des institutions financières. La mise à jour de la ligne directrice B-15 par le BSIF, notamment le report des exigences liées aux émissions de GES de portée 3, peut influencer la manière dont les banques planifient leur conformité, structurent leurs contrôles ESG et communiquent leurs risques climatiques. Ce point est important à suivre, car il permet d'évaluer l'évolution des attentes prudentielles, la comparabilité des pratiques de divulgation entre pairs et le niveau de préparation des banques face aux exigences climatiques.
-Point de surveillance : Risque climatique / ESG — Le changement indique que la banque tient compte de la mise à jour de la ligne directrice B-15 du BSIF et du report des exigences liées aux émissions de GES de portée 3. Ce point permet de suivre l'adaptation des banques aux attentes prudentielles climatiques, leur niveau de préparation ESG et la comparabilité de leurs pratiques de divulgation entre pairs.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1166,47 +1175,47 @@
       <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Activités de gestion</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Le 17 février 2025, soit le premier jour ouvrable suivant la date de rachat du 15 février 2025, la Banque a terminé le rachat de la totalité des actions privilégiées de premier rang à dividende non cumulatif à taux rajusté tous les cinq ans, série 32, émises et en circulation. Tel que prévu dans les conditions relatives aux actions, le prix de rachat était de 25,00 $ l'action, plus les dividendes périodiques déclarés et impayés. La Banque a racheté 12 000 000 actions privilégiées série 32 pour un prix total de 300 M$. Ces instruments ont été exclus du calcul des ratios de fonds propres au 31 janvier 2025.</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>Le 17 février 2025, soit le premier jour ouvrable suivant la date de rachat du 15 février 2025, la Banque a terminé le rachat de la totalité des actions privilégiées de premier rang à dividende non cumulatif à taux rajusté tous les cinq ans, série 32, émises et en circulation. Tel que prévu dans les conditions relatives aux actions, le prix de rachat était de 25,00 $ l'action, plus les dividendes périodiques déclarés et impayés. La Banque a racheté 12 000 000 actions privilégiées série 32 pour un prix total de 300 M$.</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>OUI — Nouvel élément à surveiller : Oui.
 Sujet détecté : Information retirée, fonds propres réglementaires.
@@ -1215,54 +1224,106 @@
 Point de surveillance : Fonds propres réglementaires — Le changement indique une modification de la divulgation sur la composition des fonds propres, ce qui peut affecter la comparabilité avec les pairs et la lecture des ratios de capital.</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>Non pas un vrai changement</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Risque de crédit</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Entre le 2 mars 2022 et le 12 juillet 2023, la Banque du Canada avait relevé son taux directeur à dix reprises, ce dernier passant de 0,25 % à 5 %. Cette hausse rapide des taux, qui avait pour but principal de contrer l'inflation au Canada, continue d'exercer une pression sur la capacité des titulaires d'emprunts à effectuer leurs versements, notamment celle des titulaires d'hypothèques à taux variable ou dont le terme arrive à échéance. Dans ses six dernières annonces qui ont eu lieu entre le 5 juin 2024 et le 29 janvier 2025, la Banque du Canada a abaissé son taux directeur, le faisant passer de 5 % à 3 %.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Entre le 2 mars 2022 et le 12 juillet 2023, la Banque du Canada avait relevé son taux directeur à dix reprises, ce dernier passant de 0,25 % à 5 %. Cette hausse rapide des taux, qui avait pour but principal de contrer l'inflation au Canada, continue d'exercer une pression sur la capacité des titulaires d'emprunts à effectuer leurs versements, notamment celle des titulaires d'hypothèques dont le terme est arrivé à échéance dans les derniers mois. Dans ses huit dernières annonces qui ont eu lieu entre le 5 juin 2024 et le 16 avril 2025, la Banque du Canada a abaissé son taux directeur, le faisant passer de 5 % à 2,75 %.</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>NON — Nouvel élément à surveiller : Non.
+Sujet détecté : Mise à jour quantitative propre à la banque.
+Ce qui change : Le T2 met à jour le nombre d'annonces de la Banque du Canada, passant de six à huit, et ajuste la période de référence. Ces changements sont purement factuels et ne modifient pas la substance de la divulgation.
+Pertinence métier : Cette variation ne constitue pas une nouvelle idée à surveiller, car elle reflète l'évolution normale des annonces de politique monétaire. Elle ne modifie aucun seuil prudentiel, aucune règle BSIF ou AMF, aucune méthode de calcul et aucune posture de risque qui changerait la lecture réglementaire ou la comparabilité métier.
+Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Exposition maximale au risque de crédit selon les catégories d'actifs de Bâle (1)</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Afin de respecter les exigences du BSIF en matière de divulgation relative aux prêts hypothécaires, des renseignements additionnels sont présentés dans les documents intitulés « Informations financières complémentaires - Premier trimestre 2025 » et « Informations complémentaires sur les fonds propres réglementaires et informations du Pilier 3 - Premier trimestre 2025 » disponibles sur le site Internet de la Banque à l'adresse bnc.ca.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Afin de respecter les exigences du BSIF en matière de divulgation relative aux prêts hypothécaires, des renseignements additionnels sont présentés dans les documents intitulés « Informations financières complémentaires - Deuxième trimestre 2025 » et « Informations complémentaires sur les fonds propres réglementaires et informations du Pilier 3 - Deuxième trimestre 2025 » disponibles sur le site Internet de la Banque à l'adresse bnc.ca.</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour de période de référence.
@@ -1271,50 +1332,50 @@
 Point de surveillance : Mise à jour de période — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>VaR des portefeuilles de négociation (1) (2)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>La moyenne de la VaR totale des portefeuilles de négociation a augmenté, passant de 7,9 M$ à 12,1 M$ entre le quatrième trimestre de 2024 et le premier trimestre de 2025, principalement en raison d'une hausse du risque de taux d'intérêt.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>La moyenne de la VaR totale des portefeuilles de négociation est demeurée stable entre le premier trimestre et le deuxième trimestre de 2025.</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour quantitative propre à la banque.
@@ -1323,50 +1384,102 @@
 Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Ratio de liquidité à court terme</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Le tableau de la page suivante présente les positions moyennes du LCR calculées à partir des observations quotidiennes du trimestre. Le LCR moyen de la Banque au cours du trimestre terminé le 31 janvier 2025 est de 154 %, bien au-delà de l'exigence réglementaire de 100 %, ce qui démontre que la position de liquidité à court terme de la Banque est solide.</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Le tableau de la page suivante présente les positions moyennes du LCR calculées à partir des observations quotidiennes du trimestre. Le LCR moyen de la Banque au cours du trimestre terminé le 30 avril 2025 est de 166 %, bien au-delà de l'exigence réglementaire de 100 %, ce qui démontre que la position de liquidité à court terme de la Banque est solide.</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>NON — Nouvel élément à surveiller : Non.
+Sujet détecté : Mise à jour quantitative propre à la banque.
+Ce qui change : Le T2 met à jour la date et le pourcentage du LCR moyen, passant de janvier à avril et de 154 % à 166 %. Ce changement est purement factuel et ne modifie pas la substance de la divulgation.
+Pertinence métier : Cette variation ne constitue pas une nouvelle idée à surveiller, car elle reflète l'évolution normale des mesures de liquidité propres à la banque. Elle ne modifie aucun seuil prudentiel, aucune règle BSIF ou AMF, aucune méthode de calcul et aucune posture de risque qui changerait la lecture réglementaire ou la comparabilité métier.
+Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Gestion des risques</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Exigences de déclaration relatives au ratio de liquidité à court terme (1) (2)</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Au 31 janvier 2025, les actifs liquides de niveau 1 représentent 84 % des HQLA de la Banque, qui comprennent la trésorerie, les dépôts auprès des banques centrales, les obligations émises ou garanties par le gouvernement du Canada et les gouvernements provinciaux du Canada.</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Au 30 avril 2025, les actifs liquides de niveau 1 représentent 84 % des HQLA de la Banque, qui comprennent la trésorerie, les dépôts auprès des banques centrales, les obligations émises ou garanties par le gouvernement du Canada et les gouvernements provinciaux du Canada.</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour de date de référence.
@@ -1375,50 +1488,50 @@
 Point de surveillance : Mise à jour de date — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Exigences de déclaration relatives au ratio de liquidité à court terme (1) (2)</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Les sorties de trésorerie découlent de l'application d'hypothèses, définies par le BSIF, sur les dépôts, la dette, le financement garanti, les engagements et les exigences de garanties supplémentaires. Les sorties de trésorerie sont en partie contrebalancées par les entrées de trésorerie, qui proviennent principalement de prêts garantis et de prêts performants. La Banque s'attend à ce que les LCR présentés varient d'un trimestre à l'autre, sans que ces variations ne représentent nécessairement une tendance. La variation entre le trimestre terminé le 31 janvier 2025 et le trimestre précédent découle du cours normal des activités. Les réserves de liquidités de la Banque dépassent largement le total des sorties nettes de trésorerie.</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Les sorties de trésorerie découlent de l'application d'hypothèses, définies par le BSIF, sur les dépôts, la dette, le financement garanti, les engagements et les exigences de garanties supplémentaires. Les sorties de trésorerie sont en partie contrebalancées par les entrées de trésorerie, qui proviennent principalement de prêts garantis et de prêts performants. La Banque s'attend à ce que les LCR présentés varient d'un trimestre à l'autre, sans que ces variations ne représentent nécessairement une tendance. La variation entre le trimestre terminé le 30 avril 2025 et le trimestre précédent découle du cours normal des activités. Les réserves de liquidités de la Banque dépassent largement le total des sorties nettes de trésorerie.</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour de date de référence.
@@ -1427,50 +1540,50 @@
 Point de surveillance : Mise à jour de date — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>Ratio structurel de liquidité à long terme</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Le tableau suivant présente les positions calibrées du NSFR calculées selon la stabilité des passifs et la liquidité des actifs conformément à la ligne directrice Normes de liquidité du BSIF. Le NSFR de la Banque au 31 janvier 2025 est de 123 %, bien au-delà de l'exigence réglementaire de 100 %, ce qui démontre que la position de liquidité à long terme de la Banque est solide.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Le tableau suivant présente les positions calibrées du NSFR calculées selon la stabilité des passifs et la liquidité des actifs conformément à la ligne directrice Normes de liquidité du BSIF. Le NSFR de la Banque au 30 avril 2025 est de 127 %, bien au-delà de l'exigence réglementaire de 100 %, ce qui démontre que la position de liquidité à long terme de la Banque est solide.</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour quantitative propre à la banque.
@@ -1479,50 +1592,50 @@
 Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Échéances contractuelles résiduelles des éléments du bilan et des engagements hors bilan</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Les tableaux suivants présentent les échéances contractuelles résiduelles des éléments du bilan et des engagements hors bilan au 31 janvier 2025, ainsi que les données comparatives au 31 octobre 2024. Les informations recueillies dans le cadre de cette analyse des échéances constituent une composante de la gestion des liquidités et du financement. Cependant, cette répartition par échéance n'est pas représentative de la façon dont la Banque gère son risque de taux d'intérêt, ni son risque de liquidité ni ses besoins de financement. La Banque tient compte de facteurs autres que les échéances contractuelles lorsqu'elle évalue les actifs liquides ou les flux de trésorerie futurs prévus.</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Les tableaux suivants présentent les échéances contractuelles résiduelles des éléments du bilan et des engagements hors bilan au 30 avril 2025, ainsi que les données comparatives au 31 octobre 2024. Les informations recueillies dans le cadre de cette analyse des échéances constituent une composante de la gestion des liquidités et du financement. Cependant, cette répartition par échéance n'est pas représentative de la façon dont la Banque gère son risque de taux d'intérêt, ni son risque de liquidité ni ses besoins de financement. La Banque tient compte de facteurs autres que les échéances contractuelles lorsqu'elle évalue les actifs liquides ou les flux de trésorerie futurs prévus.</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour de date de référence.
@@ -1531,50 +1644,50 @@
 Point de surveillance : Risque climatique / ESG — Le changement indique que la banque tient compte de la mise à jour de la ligne directrice B-15 du BSIF et du report des exigences liées aux émissions de GES de portée 3. Ce point permet de suivre l'adaptation des banques aux attentes prudentielles climatiques, leur niveau de préparation ESG et la comparabilité de leurs pratiques de divulgation entre pairs.</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Échéances contractuelles résiduelles des éléments du bilan et des engagements hors bilan</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>39</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>42</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
         <is>
           <t>Dans le cours normal de ses activités, la Banque prend divers engagements hors bilan. Les instruments de crédit utilisés pour répondre aux besoins de financement de ses clients représentent le montant maximal du crédit additionnel que la Banque peut devoir consentir si les engagements sont entièrement utilisés.</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>Dans le cours normal de ses activités, la Banque prend divers engagements hors bilan. Les instruments de crédit utilisés pour répondre aux besoins de financement de sa clientèle représentent le montant maximal du crédit additionnel que la Banque peut devoir consentir si les engagements sont entièrement utilisés.</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Reformulation mineure.
@@ -1583,50 +1696,50 @@
 Point de surveillance : Reformulation mineure — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="J24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Gestion des risques</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Divulgation d'information sur les risques</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>44</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>47</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>Le Rapport annuel 2024, le Rapport aux actionnaires - Premier trimestre 2025 et les documents d'informations complémentaires y afférant ont pour objectif la présentation de renseignements transparents et de grande qualité concernant les risques, conformément aux recommandations du groupe EDTF du Conseil de stabilité financière. Le tableau suivant présente un sommaire des informations relatives aux 32 recommandations du groupe EDTF ainsi que les pages de référence pour aider les utilisateurs à trouver ces informations.</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Le Rapport annuel 2024, le Rapport aux actionnaires - Deuxième trimestre 2025 et les documents d'informations complémentaires y afférant ont pour objectif la présentation de renseignements transparents et de grande qualité concernant les risques, conformément aux recommandations du groupe EDTF du Conseil de stabilité financière. Le tableau suivant présente un sommaire des informations relatives aux 32 recommandations du groupe EDTF ainsi que les pages de référence pour aider les utilisateurs à trouver ces informations.</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour de période de référence.
@@ -1635,50 +1748,102 @@
 Point de surveillance : Risque climatique / ESG — Le changement indique que la banque tient compte de la mise à jour de la ligne directrice B-15 du BSIF et du report des exigences liées aux émissions de GES de portée 3. Ce point permet de suivre l'adaptation des banques aux attentes prudentielles climatiques, leur niveau de préparation ESG et la comparabilité de leurs pratiques de divulgation entre pairs.</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Accord de Bâle</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>La ligne directrice Capacité totale d'absorption des pertes (Total Loss Absorbing Capacity ou TLAC) du BSIF, qui s'applique à toutes les BISI dans le cadre des règlements sur la recapitalisation interne du gouvernement fédéral, vise à faire en sorte qu'une BISI dispose d'une capacité d'absorption des pertes suffisante pour soutenir sa recapitalisation interne dans le cas peu probable où elle deviendrait non viable. La TLAC disponible comprend le total des fonds propres ainsi que certaines dettes de premier rang non garanties qui satisfont tous les critères d'admissibilité à la ligne directrice TLAC du BSIF. Le BSIF exige des BISI qu'elles maintiennent un ratio TLAC fondé sur les risques d'au moins 25,0 % (incluant la RSI) de l'actif pondéré en fonction des risques et un ratio de levier TLAC d'au moins 7,25 %. Le ratio TLAC se calcule en divisant la TLAC disponible par l'actif pondéré en fonction des risques et le ratio de levier TLAC se calcule en divisant la TLAC disponible par l'exposition totale. Au 31 janvier 2025, la valeur des éléments de passif en circulation faisant l'objet de règlements sur la conversion aux fins de la recapitalisation interne s'élève à 23,8 G$ (23,5 G$ au 31 octobre 2024).</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>La ligne directrice Capacité totale d'absorption des pertes (Total Loss Absorbing Capacity ou TLAC) du BSIF, qui s'applique à toutes les BISI dans le cadre des règlements sur la recapitalisation interne du gouvernement fédéral, vise à faire en sorte qu'une BISI dispose d'une capacité d'absorption des pertes suffisante pour soutenir sa recapitalisation interne dans le cas peu probable où elle deviendrait non viable. La TLAC disponible comprend le total des fonds propres ainsi que certaines dettes de premier rang non garanties qui satisfont tous les critères d'admissibilité à la ligne directrice TLAC du BSIF. Le BSIF exige des BISI qu'elles maintiennent un ratio TLAC fondé sur les risques d'au moins 25,0 % (incluant la RSI) de l'actif pondéré en fonction des risques et un ratio de levier TLAC d'au moins 7,25 %. Le ratio TLAC se calcule en divisant la TLAC disponible par l'actif pondéré en fonction des risques et le ratio de levier TLAC se calcule en divisant la TLAC disponible par l'exposition totale. Au 30 avril 2025, la valeur des éléments de passif en circulation faisant l'objet de règlements sur la conversion aux fins de la recapitalisation interne s'élève à 23,4 G$ (23,5 G$ au 31 octobre 2024).</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>NON — Nouvel élément à surveiller : Non.
+Sujet détecté : Mise à jour quantitative propre à la banque.
+Ce qui change : Le T2 met à jour la date et la valeur des éléments de passif en circulation, sans modification de fond.
+Pertinence métier : Cette variation ne constitue pas une nouvelle idée à surveiller, car elle reflète l'évolution normale d'un chiffre propre à la banque. Elle ne modifie aucun seuil prudentiel, aucune règle BSIF ou AMF, aucune méthode de calcul et aucune posture de risque qui changerait la lecture réglementaire ou la comparabilité métier.
+Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Gestion du capital</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Dividendes</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>Le 25 février 2025, le conseil d'administration a déclaré les dividendes réguliers sur les diverses séries d'actions privilégiées de premier rang, ainsi qu'un dividende de 1,14 $ par action ordinaire, payable le 1 er mai 2025 aux actionnaires inscrits le 31 mars 2025.</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>Le 27 mai 2025, le conseil d'administration a déclaré les dividendes réguliers sur les diverses séries d'actions privilégiées de premier rang, ainsi qu'un dividende de 1,18 $ par action ordinaire, en hausse de 4 cents ou 3,4 %, payable le 1 er août 2025 aux actionnaires inscrits le 30 juin 2025.</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour quantitative propre à la banque.
@@ -1687,50 +1852,50 @@
 Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Actions, autres instruments de capitaux propres et options d'achat d'actions</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>Au 21 février 2025, le nombre d'actions ordinaires en circulation se chiffre à 391 216 059 et le nombre d'options en cours est de 11 778 661.</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>Au 23 mai 2025, le nombre d'actions ordinaires en circulation se chiffre à 391 340 763 et le nombre d'options en cours est de 11 619 774.</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour quantitative propre à la banque.
@@ -1739,50 +1904,50 @@
 Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Actions, autres instruments de capitaux propres et options d'achat d'actions</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>Selon un prix-plancher de 5,00 $ et en tenant compte des dividendes et intérêts cumulés estimés, ces instruments de fonds propres assortis d'une clause FPUNV se convertiraient en un maximum de 1 264 millions d'actions ordinaires de la Banque, d'où un effet dilutif de 78,7 % selon le nombre d'actions ordinaires de la Banque en circulation au 31 janvier 2025.</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>Selon un prix-plancher de 5,00 $ et en tenant compte des dividendes et intérêts cumulés estimés, ces instruments de fonds propres assortis d'une clause FPUNV se convertiraient en un maximum de 1 472 millions d'actions ordinaires de la Banque, d'où un effet dilutif de 79,0 % selon le nombre d'actions ordinaires de la Banque en circulation au 30 avril 2025.</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour quantitative propre à la banque.
@@ -1791,50 +1956,50 @@
 Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>Ratios des fonds propres réglementaires, de levier et TLAC</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
         <is>
           <t>Le ratio des fonds propres CET1, le ratio des fonds propres de catégorie 1 et le ratio du total des fonds propres s'établissent, respectivement, à 13,6 %, à 15,5 % et à 17,1 % au 31 janvier 2025, comparativement à des ratios de 13,7 %, de 15,9 % et de 17,0 %, respectivement, au 31 octobre 2024. Le ratio des fonds propres CET1 et le ratio des fonds propres de catégorie 1 sont en baisse comparativement au 31 octobre 2024, alors que le ratio du total des fonds propres est légèrement en hausse. La croissance organique de l'actif pondéré en fonction des risques a eu un impact défavorable sur les ratios, atténué par le résultat net, déduction faite des dividendes. Le rachat d'actions privilégiées pour un montant de 300 M$ effectué le 17 février 2025, déjà exclu du calcul des ratios des fonds propres au 31 janvier 2025, a eu un impact défavorable sur le ratio des fonds propres de catégorie 1, alors que l'émission de 1,0 G$ des billets à moyen terme, le 13 janvier 2025, a eu un impact favorable sur le ratio du total des fonds propres.</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>Le ratio des fonds propres CET1, le ratio des fonds propres de catégorie 1 et le ratio du total des fonds propres s'établissent, respectivement, à 13,4 %, à 15,1 % et à 16,9 % au 30 avril 2025, comparativement à des ratios de 13,7 %, de 15,9 % et de 17,0 %, respectivement, au 31 octobre 2024. Tous les ratios des fonds propres sont en baisse comparativement au 31 octobre 2024. La croissance de l'actif pondéré en fonction des risques, principalement due à l'inclusion de CWB, a eu un impact défavorable sur les ratios, un impact atténué par les actions ordinaires émises dans le cadre de l'acquisition de CWB et par le résultat net, déduction faite des dividendes. De plus, le rachat d'actions privilégiées effectué le 17 février 2025 atténué par l'échange des actions privilégiées de CWB contre des actions privilégiées de la Banque le 20 février 2025 a eu un impact défavorable sur les ratios des fonds propres de catégorie 1 et du total des fonds propres, alors que l'émission de 1,0 G$ des billets à moyen terme, le 13 janvier 2025 et les obligations liées aux dettes subordonnées de CWB de 525 M$ ont eu un impact favorable sur le ratio du total des fonds propres.</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour quantitative propre à la banque.
@@ -1843,50 +2008,50 @@
 Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="J30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Gestion du capital</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Ratios des fonds propres réglementaires, de levier et TLAC</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>Modification</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Modification</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>Au cours du trimestre terminé le 31 janvier 2025, la Banque a respecté toutes les exigences réglementaires imposées par le BSIF en matière de capital, de levier et de TLAC.</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Au cours du trimestre et du semestre terminés le 30 avril 2025, la Banque a respecté toutes les exigences réglementaires imposées par le BSIF en matière de capital, de levier et de TLAC.</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>NON — Nouvel élément à surveiller : Non.
 Sujet détecté : Mise à jour quantitative propre à la banque.
@@ -1895,10 +2060,10 @@
 Point de surveillance : Mise à jour quantitative — La substance de la divulgation demeure stable. Ce point peut être écarté du suivi prioritaire, sauf si une autre information indique un changement de seuil prudentiel, de méthode, de conformité ou de posture de risque.</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
+      <c r="J31" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J28"/>
+  <autoFilter ref="A1:J31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>